<commit_message>
Keep sentence practice on the map and derive person from movement roll
</commit_message>
<xml_diff>
--- a/Documentatie/Opdrachtenmatrix.xlsx
+++ b/Documentatie/Opdrachtenmatrix.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overzicht" sheetId="1" r:id="R5239869a829248d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A0-A1" sheetId="2" r:id="R9c9b03563b084f63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A1-A1plus" sheetId="3" r:id="Rd6dec8b6eaaa4967"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A1-A2" sheetId="4" r:id="R937d2bffa5594e80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A2-B1" sheetId="5" r:id="R3c3dd649c6ea4736"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zinnenspel" sheetId="6" r:id="R765a11cd99c64d49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overzicht" sheetId="1" r:id="R686cf0388d13459a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A0-A1" sheetId="2" r:id="R8a8ae59c8ac14846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A1-A1plus" sheetId="3" r:id="R706f315679164bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A1-A2" sheetId="4" r:id="Raa0cbb45f7a64ed5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A2-B1" sheetId="5" r:id="R00c0b73ae37a4b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zinnenspel" sheetId="6" r:id="R92d9c52367124d1c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8292,7 +8292,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42d04694f86e463b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re26e49de5e5445cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15645,7 +15645,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32bf5a0fb08f45b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R829457d30f264a0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22998,7 +22998,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb769bc0e206a4870"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d1716647ace480e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30351,7 +30351,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8586c4dc860a4cbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5c781152a1549b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30375,7 +30375,7 @@
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Eenvoudig zinnenspel</x:v>
+        <x:v>Zinnen maken op de kaart</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
         <x:v>Eenvoudig zinnenspel</x:v>
@@ -30425,9 +30425,9 @@
         <x:v>Eenvoudig zinnenspel</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="27" customHeight="1">
+    <x:row r="3" ht="38" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Persoon + werkwoord + tijd → maak één zin. Het voorbeeld blijft verborgen tot je erop klikt.</x:v>
+        <x:v>Eén worp: de pion loopt het aantal ogen en dezelfde worp bepaalt de persoon. Het werkwoord en de tijd staan onder de kaart.</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -30539,7 +30539,7 @@
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
       <x:c r="A11" s="8" t="str">
-        <x:v>Startkeuze A0–A1: 3 personen, 6 werkwoorden, alleen groen (18 combinaties). A1–A1+: alle personen, 12 werkwoorden, groen. A1–A2: 24 werkwoorden, groen en rood. A2–B1: alle tijden. De docent kan dit aanpassen; maximaal 432 combinaties.</x:v>
+        <x:v>Op de kaart doen alle 6 personen mee. Startkeuze A0–A1: 6 werkwoorden en groen (36 combinaties). A1–A1+: 12 werkwoorden en groen. A1–A2: 24 werkwoorden, groen en rood. A2–B1: alle tijden. Kies werkwoorden en tijden bij Bord &amp; oefenen. Maximaal 432 combinaties.</x:v>
       </x:c>
       <x:c r="B11" s="8"/>
       <x:c r="C11" s="8"/>
@@ -31273,7 +31273,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d9f7c550b64045"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R710191ba6a3f4f40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>